<commit_message>
new updates for booking and records
</commit_message>
<xml_diff>
--- a/src/assets/files/toll_template.xlsx
+++ b/src/assets/files/toll_template.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="16">
   <si>
     <t xml:space="preserve">Start Date</t>
   </si>
@@ -41,16 +41,45 @@
   </si>
   <si>
     <t xml:space="preserve">End Date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18/03/2024 20:50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M7 M4 Motorway to Old Wallgrove Rd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DLC50R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16/03/2024 20:36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M5 SW Hammondville Westbound</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EKJ66M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13/03/2024 01:04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M5 SW Fairford Road Eastbound</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EIJ66F</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="d/m/yyyy"/>
-    <numFmt numFmtId="166" formatCode="m/d/yyyy"/>
+    <numFmt numFmtId="166" formatCode="[$$-409]#,##0.00;[RED]\-[$$-409]#,##0.00"/>
+    <numFmt numFmtId="167" formatCode="m/d/yyyy"/>
+    <numFmt numFmtId="168" formatCode="mm/dd/yy\ hh:mm\ AM/PM"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -118,7 +147,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -132,6 +161,18 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -152,8 +193,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
-  <sheetFormatPr defaultColWidth="12.58984375" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr defaultColWidth="12.60546875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15"/>
@@ -183,14 +224,109 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
+      <c r="A2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="G2" s="0" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B3" s="3"/>
+      <c r="A3" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>6.17</v>
+      </c>
+      <c r="G3" s="0" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>6.17</v>
+      </c>
+      <c r="G4" s="0" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6"/>
+      <c r="E5" s="5"/>
+      <c r="G5" s="6"/>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6"/>
+      <c r="E6" s="5"/>
+      <c r="G6" s="6"/>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6"/>
+      <c r="E7" s="5"/>
+      <c r="G7" s="6"/>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6"/>
+      <c r="E8" s="5"/>
+      <c r="G8" s="6"/>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6"/>
+      <c r="E9" s="5"/>
+      <c r="G9" s="6"/>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6"/>
+      <c r="E10" s="5"/>
+      <c r="G10" s="6"/>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6"/>
+      <c r="E11" s="5"/>
+      <c r="G11" s="6"/>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6"/>
+      <c r="E12" s="5"/>
+      <c r="G12" s="6"/>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6"/>
+      <c r="E13" s="5"/>
+      <c r="G13" s="6"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>